<commit_message>
feat: optimize player cards as lossless WebP
</commit_message>
<xml_diff>
--- a/configs/Datas/#Player.xlsx
+++ b/configs/Datas/#Player.xlsx
@@ -226,7 +226,7 @@
     <t>portraits/player_apex.jpg</t>
   </si>
   <si>
-    <t>player-cards/apex.png</t>
+    <t>player-cards/apex.webp</t>
   </si>
   <si>
     <t>player_flamez</t>
@@ -244,7 +244,7 @@
     <t>portraits/player_flamez.jpg</t>
   </si>
   <si>
-    <t>player-cards/flamez.png</t>
+    <t>player-cards/flamez.webp</t>
   </si>
   <si>
     <t>player_zywoo</t>
@@ -265,7 +265,7 @@
     <t>portraits/player_zywoo.jpg</t>
   </si>
   <si>
-    <t>player-cards/zywoo.png</t>
+    <t>player-cards/zywoo.webp</t>
   </si>
   <si>
     <t>player_mezii</t>
@@ -283,7 +283,7 @@
     <t>portraits/player_mezii.jpg</t>
   </si>
   <si>
-    <t>player-cards/mezii.png</t>
+    <t>player-cards/mezii.webp</t>
   </si>
   <si>
     <t>player_ropz</t>
@@ -304,7 +304,7 @@
     <t>portraits/player_ropz.jpg</t>
   </si>
   <si>
-    <t>player-cards/ropz.png</t>
+    <t>player-cards/ropz.webp</t>
   </si>
   <si>
     <t>player_kyousuke</t>
@@ -325,7 +325,7 @@
     <t>portraits/player_kyousuke.jpg</t>
   </si>
   <si>
-    <t>player-cards/kyousuke2.png</t>
+    <t>player-cards/kyousuke2.webp</t>
   </si>
   <si>
     <t>player_kyxsan</t>
@@ -340,7 +340,7 @@
     <t>portraits/player_kyxsan.jpg</t>
   </si>
   <si>
-    <t>player-cards/karrigan.png</t>
+    <t>player-cards/karrigan.webp</t>
   </si>
   <si>
     <t>player_monesy</t>
@@ -355,7 +355,7 @@
     <t>portraits/player_monesy.jpg</t>
   </si>
   <si>
-    <t>player-cards/monesy.png</t>
+    <t>player-cards/monesy.webp</t>
   </si>
   <si>
     <t>player_niko</t>
@@ -370,7 +370,7 @@
     <t>portraits/player_niko.jpg</t>
   </si>
   <si>
-    <t>player-cards/niko2.png</t>
+    <t>player-cards/niko2.webp</t>
   </si>
   <si>
     <t>player_teses</t>
@@ -391,7 +391,7 @@
     <t>portraits/player_teses.jpg</t>
   </si>
   <si>
-    <t>player-cards/TeSeS.png</t>
+    <t>player-cards/TeSeS.webp</t>
   </si>
   <si>
     <t>player_donk</t>
@@ -409,7 +409,7 @@
     <t>portraits/player_donk.jpg</t>
   </si>
   <si>
-    <t>player-cards/donk.png</t>
+    <t>player-cards/donk.webp</t>
   </si>
   <si>
     <t>player_sh1ro</t>
@@ -421,7 +421,7 @@
     <t>portraits/player_sh1ro.jpg</t>
   </si>
   <si>
-    <t>player-cards/sh1ro.png</t>
+    <t>player-cards/sh1ro.webp</t>
   </si>
   <si>
     <t>player_chopper</t>
@@ -433,7 +433,7 @@
     <t>portraits/player_chopper.jpg</t>
   </si>
   <si>
-    <t>player-cards/tn1r.png</t>
+    <t>player-cards/tn1r.webp</t>
   </si>
   <si>
     <t>player_zont1x</t>
@@ -445,7 +445,7 @@
     <t>portraits/player_zont1x.jpg</t>
   </si>
   <si>
-    <t>player-cards/zont1x.png</t>
+    <t>player-cards/zont1x.webp</t>
   </si>
   <si>
     <t>player_magixx</t>
@@ -460,7 +460,7 @@
     <t>portraits/player_magixx.jpg</t>
   </si>
   <si>
-    <t>player-cards/magixx.png</t>
+    <t>player-cards/magixx.webp</t>
   </si>
   <si>
     <t>player_b1t</t>
@@ -475,7 +475,7 @@
     <t>portraits/player_b1t.jpg</t>
   </si>
   <si>
-    <t>player-cards/b1t.png</t>
+    <t>player-cards/b1t.webp</t>
   </si>
   <si>
     <t>player_w0nderful</t>
@@ -487,7 +487,7 @@
     <t>portraits/player_w0nderful.jpg</t>
   </si>
   <si>
-    <t>player-cards/wonderful.png</t>
+    <t>player-cards/wonderful.webp</t>
   </si>
   <si>
     <t>player_im</t>
@@ -502,7 +502,7 @@
     <t>portraits/player_im.jpg</t>
   </si>
   <si>
-    <t>player-cards/im.png</t>
+    <t>player-cards/im.webp</t>
   </si>
   <si>
     <t>player_aleksib</t>
@@ -514,7 +514,7 @@
     <t>portraits/player_aleksib.jpg</t>
   </si>
   <si>
-    <t>player-cards/aleksib.png</t>
+    <t>player-cards/aleksib.webp</t>
   </si>
   <si>
     <t>player_makazze</t>
@@ -529,7 +529,7 @@
     <t>portraits/player_makazze.jpg</t>
   </si>
   <si>
-    <t>player-cards/makazee.png</t>
+    <t>player-cards/makazee.webp</t>
   </si>
 </sst>
 </file>

</xml_diff>